<commit_message>
deploy: main → 01ba86602f9ecfb1c6e3153aae0da551cc1987b9
</commit_message>
<xml_diff>
--- a/StructureDefinition-SEEHDSLMObservationsV12.xlsx
+++ b/StructureDefinition-SEEHDSLMObservationsV12.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4919" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4919" uniqueCount="415">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-15T17:10:15+00:00</t>
+    <t>2026-10-15T18:03:33+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -371,7 +371,10 @@
 </t>
   </si>
   <si>
-    <t>rivId</t>
+    <t>Id för patienten, 12 tecken utan avskiljare (IIType)</t>
+  </si>
+  <si>
+    <t>- root: OID för typ av identifierare. Personnummer 1.2.752.129.2.1.3.1, samordningsnummer 1.2.752.129.2.1.3.3, reservnummer lokalt definierad OID (t.ex. SLL reservnummer 1.2.752.97.3.1.3). - extension: personnummer/samordningsnummer/reservnummer.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.patient.name</t>
@@ -381,7 +384,10 @@
 </t>
   </si>
   <si>
-    <t>name</t>
+    <t>Personens namn</t>
+  </si>
+  <si>
+    <t>Personens namn.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.patient.dateOfBirth</t>
@@ -391,10 +397,11 @@
 </t>
   </si>
   <si>
-    <t>dateOfBirth</t>
-  </si>
-  <si>
-    <t>Format enligt XSD (DateType): ÅÅÅÅMMDD.</t>
+    <t>Patientens födelseår, månad och dag. Ej personnummer. Format ÅÅÅÅMMDD (DateType)</t>
+  </si>
+  <si>
+    <t>Patientens födelseår, månad och dag. Ej personnummer. Format ÅÅÅÅMMDD (DateType).
+Format enligt XSD (DateType): ÅÅÅÅMMDD.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.patient.gender</t>
@@ -404,7 +411,10 @@
 </t>
   </si>
   <si>
-    <t>gender</t>
+    <t>Patientens kön (CVType). KV kön, OID 1.2.752.129.2.2.1.1</t>
+  </si>
+  <si>
+    <t>Koder: 0 okänt, 1 man, 2 kvinna, 9 ej tillämpligt. Kodverket finns i [R9].</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole</t>
@@ -432,16 +442,28 @@
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.rivId</t>
   </si>
   <si>
+    <t>HSA-id för personen som utfört observationen (IIType). Regel 2.1</t>
+  </si>
+  <si>
+    <t>Anges enbart om observationen utförts av hälso- och sjukvårdspersonal. root = 1.2.752.129.2.1.4.1 (HSA-katalogen), extension = HSA-id.</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.code</t>
   </si>
   <si>
-    <t>code</t>
+    <t>Den roll som utföraren agerar i under observationen (CVType)</t>
+  </si>
+  <si>
+    <t>Den roll som utföraren agerar i under observationen (CVType).</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.person</t>
   </si>
   <si>
-    <t>person</t>
+    <t>Den person som utfört observationen (PersonType). Regel 2.1</t>
+  </si>
+  <si>
+    <t>Används då det finns behov av att beskriva egenskaper hos personen som inte beskrivs i performerRole (t.ex. namn på hälso- och sjukvårdspersonal), eller då observationen utförts av en person som inte klassas som hälso- och sjukvårdspersonal.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.person.id</t>
@@ -456,13 +478,28 @@
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.person.rivId</t>
   </si>
   <si>
+    <t>Identifierare för personen (IIType)</t>
+  </si>
+  <si>
+    <t>Anges endast om observationen utförts av person som INTE klassas som hälso- och sjukvårdspersonal. root: OID för personnummer (1.2.752.129.2.1.3.1), samordningsnummer (1.2.752.129.2.1.3.3) eller lokalt definierat reservnummer. extension: personnummer/samordningsnummer/reservnummer.</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.person.name</t>
   </si>
   <si>
+    <t>För- och efternamn i klartext. Regel 2.1</t>
+  </si>
+  <si>
+    <t>För- och efternamn i klartext. Regel 2.1.</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.careUnit</t>
   </si>
   <si>
-    <t>careUnit</t>
+    <t>PDL-vårdenhet och vårdgivare som observationen utförs på uppdrag av (CareUnitType). Regel 2.1, 2.5</t>
+  </si>
+  <si>
+    <t>Ska endast anges då den person som utfört observationen är hälso- och sjukvårdspersonal. Krävs för spärrhantering, åtkomstkontroll samt loggning enligt PDL.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.careUnit.id</t>
@@ -477,13 +514,28 @@
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.careUnit.rivId</t>
   </si>
   <si>
+    <t>HSA-id för PDL-vårdenhet med medicinskt ansvar för observationen (IIType)</t>
+  </si>
+  <si>
+    <t>HSA-id för PDL-vårdenhet med medicinskt ansvar för observationen (IIType).</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.careUnit.name</t>
   </si>
   <si>
+    <t>Vårdenhetens namn</t>
+  </si>
+  <si>
+    <t>Vårdenhetens namn.</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.careUnit.careGiver</t>
   </si>
   <si>
-    <t>careGiver</t>
+    <t>Den vårdgivare som enheten är knuten till (CareGiverType)</t>
+  </si>
+  <si>
+    <t>Den vårdgivare som enheten är knuten till (CareGiverType).</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.careUnit.careGiver.id</t>
@@ -498,9 +550,21 @@
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.careUnit.careGiver.rivId</t>
   </si>
   <si>
+    <t>HSA-id för vårdgivaren (IIType)</t>
+  </si>
+  <si>
+    <t>HSA-id för vårdgivaren (IIType).</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.performerRole.careUnit.careGiver.name</t>
   </si>
   <si>
+    <t>Vårdgivarens namn</t>
+  </si>
+  <si>
+    <t>Vårdgivarens namn.</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.legalAuthenticator</t>
   </si>
   <si>
@@ -520,6 +584,12 @@
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.legalAuthenticator.rivId</t>
+  </si>
+  <si>
+    <t>HSA-id för personen som signerat (IIType). root = 1.2.752.129.2.1.4.1</t>
+  </si>
+  <si>
+    <t>HSA-id för personen som signerat (IIType). root = 1.2.752.129.2.1.4.1.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.legalAuthenticator.time</t>
@@ -529,10 +599,19 @@
 </t>
   </si>
   <si>
-    <t>YYYY, YYYYMM, YYYYMMDD, YYYYMMDDhh, YYYYMMDDhhmm, YYYYMMDDhhmmss</t>
+    <t>Tid för signeringen (PartialTimeStampType). Format ÅÅÅÅMMDDttmmss där klockslaget är frivilligt</t>
+  </si>
+  <si>
+    <t>Tid för signeringen (PartialTimeStampType). Format ÅÅÅÅMMDDttmmss där klockslaget är frivilligt.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.legalAuthenticator.name</t>
+  </si>
+  <si>
+    <t>För- och efternamn i klartext för signerande person. Regel 2.3</t>
+  </si>
+  <si>
+    <t>För- och efternamn i klartext för signerande person. Regel 2.3.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant</t>
@@ -560,16 +639,25 @@
     <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.rivId</t>
   </si>
   <si>
+    <t>HSA-id för ytterligare deltagare som är hälso- och sjukvårdspersonal (IIType)</t>
+  </si>
+  <si>
+    <t>HSA-id för ytterligare deltagare som är hälso- och sjukvårdspersonal (IIType).</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.type</t>
   </si>
   <si>
-    <t>type</t>
+    <t>Typ av deltagande (CVType), t.ex. sekundär utförare/assistent</t>
+  </si>
+  <si>
+    <t>codeSystemName, codeSystemVersion och displayName ska ej anges (0..0).</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.role</t>
   </si>
   <si>
-    <t>role</t>
+    <t>Den roll deltagaren agerar i (CVType), t.ex. anhörig eller vårdpersonal</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.time</t>
@@ -579,243 +667,372 @@
 </t>
   </si>
   <si>
+    <t>Deltagandetid om den inte överensstämmer med observationens (TimePeriodType)</t>
+  </si>
+  <si>
+    <t>Deltagandetid om den inte överensstämmer med observationens (TimePeriodType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person</t>
+  </si>
+  <si>
+    <t>Deltagande övrig person (PersonType)</t>
+  </si>
+  <si>
+    <t>Deltagande övrig person (PersonType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.rivId</t>
+  </si>
+  <si>
+    <t>Identifierare för personen (IIType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.name</t>
+  </si>
+  <si>
+    <t>För- och efternamn i klartext</t>
+  </si>
+  <si>
+    <t>För- och efternamn i klartext.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation</t>
+  </si>
+  <si>
+    <t>Deltagande övrig organisation (OrganisationType)</t>
+  </si>
+  <si>
+    <t>Deltagande övrig organisation (OrganisationType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.rivId</t>
+  </si>
+  <si>
+    <t>Id för organisation, vanligtvis HSA-id (root 1.2.752.129.2.1.4.1)</t>
+  </si>
+  <si>
+    <t>Id för organisation, vanligtvis HSA-id (root 1.2.752.129.2.1.4.1).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.name</t>
+  </si>
+  <si>
+    <t>Organisationens namn</t>
+  </si>
+  <si>
+    <t>Organisationens namn.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device</t>
+  </si>
+  <si>
+    <t>Deltagande utrustning (DeviceType)</t>
+  </si>
+  <si>
+    <t>Deltagande utrustning (DeviceType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.rivId</t>
+  </si>
+  <si>
+    <t>Identitetsbeteckning på en viss verklig instans av utrustning (IIType)</t>
+  </si>
+  <si>
+    <t>Identitetsbeteckning på en viss verklig instans av utrustning (IIType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.type</t>
+  </si>
+  <si>
+    <t>Typ av deltagande utrustning (CVType)</t>
+  </si>
+  <si>
+    <t>Typ av deltagande utrustning (CVType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model</t>
+  </si>
+  <si>
+    <t>Modell för angiven utrustning (SCType)</t>
+  </si>
+  <si>
+    <t>Modell för angiven utrustning (SCType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.code</t>
+  </si>
+  <si>
+    <t>Modellbeteckning (CVType). codeSystemVersion ska ej anges</t>
+  </si>
+  <si>
+    <t>Modellbeteckning (CVType). codeSystemVersion ska ej anges.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.value</t>
+  </si>
+  <si>
+    <t>Tillverkarens modellbeteckning i klartext; komplement eller i stället för modelCode</t>
+  </si>
+  <si>
+    <t>Tillverkarens modellbeteckning i klartext; komplement eller i stället för modelCode.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location</t>
+  </si>
+  <si>
+    <t>Deltagande plats (LocationType). Sammanslagning av roll och plats enligt V-MIM</t>
+  </si>
+  <si>
+    <t>Deltagande plats (LocationType). Sammanslagning av roll och plats enligt V-MIM.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.rivId</t>
+  </si>
+  <si>
+    <t>HSA-id för platsen; anges om platsen är en vårdenhet (IIType)</t>
+  </si>
+  <si>
+    <t>HSA-id för platsen; anges om platsen är en vårdenhet (IIType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.name</t>
+  </si>
+  <si>
+    <t>Namn på den plats där observationen har genomförts</t>
+  </si>
+  <si>
+    <t>Namn på den plats där observationen har genomförts.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address</t>
+  </si>
+  <si>
+    <t>Adress till plats (AddressType)</t>
+  </si>
+  <si>
+    <t>Adress till plats (AddressType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.use</t>
+  </si>
+  <si>
+    <t>Adressens användning (PostalAddressUseEnum). Den primära adressen anges utan use-kod</t>
+  </si>
+  <si>
+    <t>Adressens användning (PostalAddressUseEnum). Den primära adressen anges utan use-kod.
+Tillåtna värden enligt XSD: PHYS, H, HV, WP, TMP.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part</t>
+  </si>
+  <si>
+    <t>Adressdel (AddressPartType). Delarna listas i ordningen CAR, POB, SAL, ZIP, CTY, CNT, PRE, CPA</t>
+  </si>
+  <si>
+    <t>Adressdel (AddressPartType). Delarna listas i ordningen CAR, POB, SAL, ZIP, CTY, CNT, PRE, CPA.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.value</t>
+  </si>
+  <si>
+    <t>Adressdelens värde</t>
+  </si>
+  <si>
+    <t>Adressdelens värde.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.type</t>
+  </si>
+  <si>
+    <t>Typ av adressdel (AddressPartTypeEnum, baserad på ISO 21090)</t>
+  </si>
+  <si>
+    <t>Typ av adressdel (AddressPartTypeEnum, baserad på ISO 21090).
+Tillåtna värden enligt XSD: SAL, CAR, CEN, CNT, CPA, CTY, POB, ZIP, PRE, STA.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress</t>
+  </si>
+  <si>
+    <t>Elektronisk adress till plats (TelType)</t>
+  </si>
+  <si>
+    <t>Elektronisk adress till plats (TelType).</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.use</t>
+  </si>
+  <si>
+    <t>Typ av elektronisk adress (TelTypeEnum): voice, fax, data, sms</t>
+  </si>
+  <si>
+    <t>Typ av elektronisk adress (TelTypeEnum): voice, fax, data, sms.
+Tillåtna värden enligt XSD: voice, fax, data, sms.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.value</t>
+  </si>
+  <si>
+    <t>Elektronisk adress</t>
+  </si>
+  <si>
+    <t>Elektronisk adress.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem</t>
+  </si>
+  <si>
+    <t>Källsystem som observationsgruppen lagras i</t>
+  </si>
+  <si>
+    <t>Källsystem som observationsgruppen lagras i.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem.rivId</t>
+  </si>
+  <si>
+    <t>HSA-id för källsystemet (IIType). root = 1.2.752.129.2.1.4.1</t>
+  </si>
+  <si>
+    <t>HSA-id för källsystemet (IIType). root = 1.2.752.129.2.1.4.1.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.observation</t>
+  </si>
+  <si>
+    <t>De observationer som ligger inom denna grupp av observationer</t>
+  </si>
+  <si>
+    <t>De observationer som ligger inom denna grupp av observationer.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.observation.id</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.observation.extension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.observation.modifierExtension</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.observation.rivId</t>
+  </si>
+  <si>
+    <t>Unik identifierare för observationen (IIType)</t>
+  </si>
+  <si>
+    <t>Identifieraren ska vara konsistent och beständig mellan olika majorversioner av ett kontrakt och mellan olika kontrakt. root: vårdgivarens HSA-id. extension: den inom vårdgivaren eller källsystemet unika identifieraren för observationen.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.observation.type</t>
+  </si>
+  <si>
+    <t>NI 2015:1 Observation.typ — kod för typ av observation (CVType)</t>
+  </si>
+  <si>
+    <t>Det som faktiskt är avsett, önskat eller observerat tillstånd dokumenteras i value. Exempelvis kan type vara "diagnos", vilket innebär att value håller diagnosen.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.observation.status</t>
+  </si>
+  <si>
+    <t>NI 2015:1 Observation.status (CVType). TKB: 0..0</t>
+  </si>
+  <si>
+    <t>Denna version av specifikationen tillåter endast faktiskt utförda observationer; TKB anger kardinalitet 0..0 medan schemat tillåter 0..1. Om statuskoden utelämnas antas detta vara en faktisk observation.</t>
+  </si>
+  <si>
+    <t>SEEHDSLMObservationsV12.observationGroup.observation.time</t>
+  </si>
+  <si>
     <t>Används för att specificera ett datumintervall med hjälp av start- och slutdatum</t>
   </si>
   <si>
     <t>Används för att specificera ett datumintervall med hjälp av start- och slutdatum. start: Startdatum på formatet YYYYMMDDhhmmss end: Slutdatum på formatet YYYYMMDDhhmmss</t>
   </si>
   <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.rivId</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.person.name</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation</t>
-  </si>
-  <si>
-    <t>organisation</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.rivId</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.organisation.name</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device</t>
-  </si>
-  <si>
-    <t>device</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.rivId</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.type</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model</t>
-  </si>
-  <si>
-    <t>model</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.code</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.device.model.value</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location</t>
-  </si>
-  <si>
-    <t>location</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.rivId</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.name</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address</t>
-  </si>
-  <si>
-    <t>address</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.use</t>
-  </si>
-  <si>
-    <t>use</t>
-  </si>
-  <si>
-    <t>Tillåtna värden enligt XSD: PHYS, H, HV, WP, TMP.</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part</t>
-  </si>
-  <si>
-    <t>part</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.value</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.address.part.type</t>
-  </si>
-  <si>
-    <t>Tillåtna värden enligt XSD: SAL, CAR, CEN, CNT, CPA, CTY, POB, ZIP, PRE, STA.</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress</t>
-  </si>
-  <si>
-    <t>electronicAddress</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.use</t>
-  </si>
-  <si>
-    <t>Tillåtna värden enligt XSD: voice, fax, data, sms.</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.additionalParticipant.location.electronicAddress.value</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem</t>
-  </si>
-  <si>
-    <t>Källsystem som observationsgruppen lagras i</t>
-  </si>
-  <si>
-    <t>Källsystem som observationsgruppen lagras i.</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.sourceSystem.rivId</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.observation</t>
-  </si>
-  <si>
-    <t>De observationer som ligger inom denna grupp av observationer</t>
-  </si>
-  <si>
-    <t>De observationer som ligger inom denna grupp av observationer.</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.observation.id</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.observation.extension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.observation.modifierExtension</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.observation.rivId</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.observation.type</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.observation.status</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>SEEHDSLMObservationsV12.observationGroup.observation.time</t>
-  </si>
-  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.time.id</t>
   </si>
   <si>
@@ -828,16 +1045,28 @@
     <t>SEEHDSLMObservationsV12.observationGroup.observation.time.start</t>
   </si>
   <si>
+    <t>YYYY, YYYYMM, YYYYMMDD, YYYYMMDDhh, YYYYMMDDhhmm, YYYYMMDDhhmmss</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.time.end</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.method</t>
   </si>
   <si>
-    <t>method</t>
+    <t>Kod för typ av tillvägagångssätt för genomförandet av observationen (CVType)</t>
+  </si>
+  <si>
+    <t>Kod för typ av tillvägagångssätt för genomförandet av observationen (CVType).</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.value</t>
+  </si>
+  <si>
+    <t>NI 2015:1 Observation.värde — observationens utfall (ValueANYType)</t>
+  </si>
+  <si>
+    <t>En och endast en av huvudtyperna cv, pq, ivl_pq, ts och ivl_ts. I schemat en xs:sequence av valfria element (av kompatibilitetsskäl i stället för xs:choice).</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.value.id</t>
@@ -856,12 +1085,21 @@
 </t>
   </si>
   <si>
-    <t>pq</t>
+    <t>Mätvärde (PQType), t.ex. 187 cm</t>
+  </si>
+  <si>
+    <t>Mätvärde (PQType), t.ex. 187 cm.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.value.ts</t>
   </si>
   <si>
+    <t>Tidpunkt (PartialTimeStampType), precision ner till endast årtal</t>
+  </si>
+  <si>
+    <t>Tidpunkt (PartialTimeStampType), precision ner till endast årtal.</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.value.ivlTs</t>
   </si>
   <si>
@@ -883,7 +1121,10 @@
     <t>SEEHDSLMObservationsV12.observationGroup.observation.value.cv</t>
   </si>
   <si>
-    <t>cv</t>
+    <t>Kodat värde (CVType), t.ex. diagnoskod enligt ICD-10 eller kliniskt fynd enligt Snomed CT</t>
+  </si>
+  <si>
+    <t>Kodat värde (CVType), t.ex. diagnoskod enligt ICD-10 eller kliniskt fynd enligt Snomed CT.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.value.ivlPq</t>
@@ -899,7 +1140,10 @@
     <t>SEEHDSLMObservationsV12.observationGroup.observation.targetSite</t>
   </si>
   <si>
-    <t>targetSite</t>
+    <t>NI 2015:1 Observation.lokalisation (CVType)</t>
+  </si>
+  <si>
+    <t>Beskriver vad observationen avser gällande anatomi, funktion eller system. Används endast om inte type innefattar tillräcklig information om detta.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.valueNegation</t>
@@ -909,19 +1153,28 @@
 </t>
   </si>
   <si>
-    <t>valueNegation</t>
+    <t>NI 2015:1 Observation.negation — negerar betydelsen av value. Normalvärde false</t>
+  </si>
+  <si>
+    <t>NI 2015:1 Observation.negation — negerar betydelsen av value. Normalvärde false.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.description</t>
   </si>
   <si>
-    <t>description</t>
+    <t>Fritextbeskrivning av observationen där sådan kompletterar kodbeteckningen</t>
+  </si>
+  <si>
+    <t>Fritextbeskrivning av observationen där sådan kompletterar kodbeteckningen.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.approvedForPatient</t>
   </si>
   <si>
-    <t>approvedForPatient</t>
+    <t>Om informationen får delas till patient (menprövad)</t>
+  </si>
+  <si>
+    <t>Om informationen får delas till patient (menprövad).</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.registrationTime</t>
@@ -931,16 +1184,20 @@
 </t>
   </si>
   <si>
-    <t>registrationTime</t>
-  </si>
-  <si>
-    <t>Format enligt XSD (TimeStampType): ÅÅÅÅMMDDttmmss.</t>
+    <t>Dokumentationstidpunkt i patientens journal. Format ÅÅÅÅMMDDttmmss (TimeStampType)</t>
+  </si>
+  <si>
+    <t>Dokumentationstidpunkt i patientens journal. Format ÅÅÅÅMMDDttmmss (TimeStampType).
+Format enligt XSD (TimeStampType): ÅÅÅÅMMDDttmmss.</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation</t>
   </si>
   <si>
-    <t>relation</t>
+    <t>Typade samband till andra informationsmängder (RelationType)</t>
+  </si>
+  <si>
+    <t>Typade samband till andra informationsmängder (RelationType).</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.id</t>
@@ -955,10 +1212,19 @@
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.code</t>
   </si>
   <si>
+    <t>Typ av relation den refererade informationen har till observationen (CVType)</t>
+  </si>
+  <si>
+    <t>Typ av relation den refererade informationen har till observationen (CVType).</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.referredInformation</t>
   </si>
   <si>
-    <t>referredInformation</t>
+    <t>Den refererade informationen (ReferredInformationType)</t>
+  </si>
+  <si>
+    <t>Den refererade informationen (ReferredInformationType).</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.referredInformation.id</t>
@@ -973,16 +1239,37 @@
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.referredInformation.rivId</t>
   </si>
   <si>
+    <t>Den refererade informationens identitet (IIType)</t>
+  </si>
+  <si>
+    <t>root: HSA-id för källsystem där den refererade informationen är lagrad. extension: ett inom vårdgivaren unikt id.</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.referredInformation.time</t>
   </si>
   <si>
+    <t>Starttid för refererad information (PartialTimeStampType). Regel 2.4</t>
+  </si>
+  <si>
+    <t>Starttid för refererad information (PartialTimeStampType). Regel 2.4.</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.referredInformation.type</t>
   </si>
   <si>
+    <t>Typ av uppgift som sambandet pekar ut — kod från Categorization i engagemangsindex, t.ex. chb-o</t>
+  </si>
+  <si>
+    <t>Typ av uppgift som sambandet pekar ut — kod från Categorization i engagemangsindex, t.ex. chb-o.</t>
+  </si>
+  <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.referredInformation.informationOwner</t>
   </si>
   <si>
-    <t>informationOwner</t>
+    <t>Vårdgivare som är informationsägare av den refererade informationen (InformationOwnerType)</t>
+  </si>
+  <si>
+    <t>Vårdgivare som är informationsägare av den refererade informationen (InformationOwnerType).</t>
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.referredInformation.informationOwner.id</t>
@@ -995,6 +1282,12 @@
   </si>
   <si>
     <t>SEEHDSLMObservationsV12.observationGroup.observation.relation.referredInformation.informationOwner.rivId</t>
+  </si>
+  <si>
+    <t>Vårdgivarens HSA-id (IIType). root = 1.2.752.129.2.1.4.1</t>
+  </si>
+  <si>
+    <t>Vårdgivarens HSA-id (IIType). root = 1.2.752.129.2.1.4.1.</t>
   </si>
 </sst>
 </file>
@@ -2392,7 +2685,7 @@
         <v>114</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2460,10 +2753,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2486,13 +2779,13 @@
         <v>72</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2543,7 +2836,7 @@
         <v>72</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>73</v>
@@ -2560,10 +2853,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2586,13 +2879,13 @@
         <v>72</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -2643,7 +2936,7 @@
         <v>72</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>83</v>
@@ -2660,10 +2953,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2686,13 +2979,13 @@
         <v>72</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2743,7 +3036,7 @@
         <v>72</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>73</v>
@@ -2760,10 +3053,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -2789,10 +3082,10 @@
         <v>78</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2843,7 +3136,7 @@
         <v>72</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>83</v>
@@ -2855,15 +3148,15 @@
         <v>72</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2960,10 +3253,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3062,10 +3355,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3166,10 +3459,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3195,10 +3488,10 @@
         <v>113</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -3249,7 +3542,7 @@
         <v>72</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>73</v>
@@ -3266,10 +3559,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3292,13 +3585,13 @@
         <v>72</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -3349,7 +3642,7 @@
         <v>72</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>83</v>
@@ -3366,10 +3659,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3395,10 +3688,10 @@
         <v>78</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3449,7 +3742,7 @@
         <v>72</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>73</v>
@@ -3466,10 +3759,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3566,10 +3859,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3668,10 +3961,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3772,10 +4065,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3801,10 +4094,10 @@
         <v>113</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>114</v>
+        <v>149</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3855,7 +4148,7 @@
         <v>72</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>73</v>
@@ -3872,10 +4165,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -3898,13 +4191,13 @@
         <v>72</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>117</v>
+        <v>152</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
@@ -3955,7 +4248,7 @@
         <v>72</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>73</v>
@@ -3972,10 +4265,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4001,10 +4294,10 @@
         <v>78</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4055,7 +4348,7 @@
         <v>72</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>73</v>
@@ -4072,10 +4365,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4172,10 +4465,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4274,10 +4567,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4378,10 +4671,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4407,10 +4700,10 @@
         <v>113</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>114</v>
+        <v>160</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4461,7 +4754,7 @@
         <v>72</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>83</v>
@@ -4478,10 +4771,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4504,13 +4797,13 @@
         <v>72</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>117</v>
+        <v>163</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>117</v>
+        <v>164</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4561,7 +4854,7 @@
         <v>72</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>73</v>
@@ -4578,10 +4871,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -4607,10 +4900,10 @@
         <v>78</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -4661,7 +4954,7 @@
         <v>72</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>83</v>
@@ -4678,10 +4971,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4778,10 +5071,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4880,10 +5173,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -4984,10 +5277,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5013,10 +5306,10 @@
         <v>113</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>114</v>
+        <v>172</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>114</v>
+        <v>173</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -5067,7 +5360,7 @@
         <v>72</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>83</v>
@@ -5084,10 +5377,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5110,13 +5403,13 @@
         <v>72</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>117</v>
+        <v>175</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>117</v>
+        <v>176</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5167,7 +5460,7 @@
         <v>72</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>73</v>
@@ -5184,10 +5477,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5213,10 +5506,10 @@
         <v>78</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -5267,7 +5560,7 @@
         <v>72</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>73</v>
@@ -5284,10 +5577,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>159</v>
+        <v>180</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>159</v>
+        <v>180</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5384,10 +5677,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -5486,10 +5779,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -5590,10 +5883,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -5619,10 +5912,10 @@
         <v>113</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>114</v>
+        <v>184</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>114</v>
+        <v>185</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -5673,7 +5966,7 @@
         <v>72</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>73</v>
@@ -5690,10 +5983,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -5716,13 +6009,13 @@
         <v>72</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>165</v>
+        <v>189</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -5773,7 +6066,7 @@
         <v>72</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>83</v>
@@ -5790,10 +6083,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -5816,13 +6109,13 @@
         <v>72</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>117</v>
+        <v>191</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>117</v>
+        <v>192</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -5873,7 +6166,7 @@
         <v>72</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>73</v>
@@ -5890,10 +6183,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>167</v>
+        <v>193</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>167</v>
+        <v>193</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -5919,10 +6212,10 @@
         <v>78</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>168</v>
+        <v>194</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>169</v>
+        <v>195</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -5973,7 +6266,7 @@
         <v>72</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>167</v>
+        <v>193</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>73</v>
@@ -5985,15 +6278,15 @@
         <v>72</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>170</v>
+        <v>196</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6090,10 +6383,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6192,10 +6485,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -6296,10 +6589,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>174</v>
+        <v>200</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>174</v>
+        <v>200</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -6325,10 +6618,10 @@
         <v>113</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>114</v>
+        <v>201</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>114</v>
+        <v>202</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -6379,7 +6672,7 @@
         <v>72</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>174</v>
+        <v>200</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>73</v>
@@ -6396,10 +6689,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>175</v>
+        <v>203</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>175</v>
+        <v>203</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -6422,13 +6715,13 @@
         <v>72</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>176</v>
+        <v>204</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>176</v>
+        <v>205</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -6479,7 +6772,7 @@
         <v>72</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>175</v>
+        <v>203</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>83</v>
@@ -6496,10 +6789,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>177</v>
+        <v>206</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>177</v>
+        <v>206</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -6522,13 +6815,13 @@
         <v>72</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>178</v>
+        <v>207</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>178</v>
+        <v>205</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
@@ -6579,7 +6872,7 @@
         <v>72</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>177</v>
+        <v>206</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>83</v>
@@ -6596,10 +6889,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>179</v>
+        <v>208</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>179</v>
+        <v>208</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -6622,13 +6915,13 @@
         <v>72</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>181</v>
+        <v>210</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>182</v>
+        <v>211</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -6679,7 +6972,7 @@
         <v>72</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>179</v>
+        <v>208</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>73</v>
@@ -6696,10 +6989,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>183</v>
+        <v>212</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>183</v>
+        <v>212</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -6725,10 +7018,10 @@
         <v>78</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>136</v>
+        <v>213</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>136</v>
+        <v>214</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -6779,7 +7072,7 @@
         <v>72</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>183</v>
+        <v>212</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>73</v>
@@ -6796,10 +7089,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>184</v>
+        <v>215</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>184</v>
+        <v>215</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -6896,10 +7189,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>185</v>
+        <v>216</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>185</v>
+        <v>216</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -6998,10 +7291,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>186</v>
+        <v>217</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>186</v>
+        <v>217</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -7102,10 +7395,10 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>187</v>
+        <v>218</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>187</v>
+        <v>218</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -7131,10 +7424,10 @@
         <v>113</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>114</v>
+        <v>219</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -7185,7 +7478,7 @@
         <v>72</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>187</v>
+        <v>218</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>73</v>
@@ -7202,10 +7495,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>188</v>
+        <v>220</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>188</v>
+        <v>220</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -7228,13 +7521,13 @@
         <v>72</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>117</v>
+        <v>221</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>117</v>
+        <v>222</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -7285,7 +7578,7 @@
         <v>72</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>188</v>
+        <v>220</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>73</v>
@@ -7302,10 +7595,10 @@
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>189</v>
+        <v>223</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>189</v>
+        <v>223</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -7331,10 +7624,10 @@
         <v>78</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>190</v>
+        <v>224</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>190</v>
+        <v>225</v>
       </c>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
@@ -7385,7 +7678,7 @@
         <v>72</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>189</v>
+        <v>223</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>73</v>
@@ -7402,10 +7695,10 @@
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>191</v>
+        <v>226</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>191</v>
+        <v>226</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -7502,10 +7795,10 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>192</v>
+        <v>227</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>192</v>
+        <v>227</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -7604,10 +7897,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>193</v>
+        <v>228</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>193</v>
+        <v>228</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -7708,10 +8001,10 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>194</v>
+        <v>229</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>194</v>
+        <v>229</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -7737,10 +8030,10 @@
         <v>113</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>114</v>
+        <v>230</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>114</v>
+        <v>231</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -7791,7 +8084,7 @@
         <v>72</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>194</v>
+        <v>229</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>73</v>
@@ -7808,10 +8101,10 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>195</v>
+        <v>232</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>195</v>
+        <v>232</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -7834,13 +8127,13 @@
         <v>72</v>
       </c>
       <c r="K65" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>117</v>
+        <v>233</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>117</v>
+        <v>234</v>
       </c>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
@@ -7891,7 +8184,7 @@
         <v>72</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>195</v>
+        <v>232</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>73</v>
@@ -7908,10 +8201,10 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
-        <v>196</v>
+        <v>235</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>196</v>
+        <v>235</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -7937,10 +8230,10 @@
         <v>78</v>
       </c>
       <c r="L66" t="s" s="2">
-        <v>197</v>
+        <v>236</v>
       </c>
       <c r="M66" t="s" s="2">
-        <v>197</v>
+        <v>237</v>
       </c>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
@@ -7991,7 +8284,7 @@
         <v>72</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>196</v>
+        <v>235</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>73</v>
@@ -8008,10 +8301,10 @@
     </row>
     <row r="67">
       <c r="A67" t="s" s="2">
-        <v>198</v>
+        <v>238</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>198</v>
+        <v>238</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -8108,10 +8401,10 @@
     </row>
     <row r="68">
       <c r="A68" t="s" s="2">
-        <v>199</v>
+        <v>239</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>199</v>
+        <v>239</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -8210,10 +8503,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -8314,10 +8607,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -8343,10 +8636,10 @@
         <v>113</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>114</v>
+        <v>242</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>114</v>
+        <v>243</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
@@ -8397,7 +8690,7 @@
         <v>72</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>73</v>
@@ -8414,10 +8707,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>202</v>
+        <v>244</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>202</v>
+        <v>244</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -8440,13 +8733,13 @@
         <v>72</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>176</v>
+        <v>245</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>176</v>
+        <v>246</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -8497,7 +8790,7 @@
         <v>72</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>202</v>
+        <v>244</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>73</v>
@@ -8514,10 +8807,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>203</v>
+        <v>247</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>203</v>
+        <v>247</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -8543,10 +8836,10 @@
         <v>78</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>204</v>
+        <v>249</v>
       </c>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
@@ -8597,7 +8890,7 @@
         <v>72</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>203</v>
+        <v>247</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>73</v>
@@ -8614,10 +8907,10 @@
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -8714,10 +9007,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>206</v>
+        <v>251</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>206</v>
+        <v>251</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -8816,10 +9109,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>207</v>
+        <v>252</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>207</v>
+        <v>252</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -8920,10 +9213,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>208</v>
+        <v>253</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>208</v>
+        <v>253</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -8946,13 +9239,13 @@
         <v>72</v>
       </c>
       <c r="K76" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L76" t="s" s="2">
-        <v>134</v>
+        <v>254</v>
       </c>
       <c r="M76" t="s" s="2">
-        <v>134</v>
+        <v>255</v>
       </c>
       <c r="N76" s="2"/>
       <c r="O76" s="2"/>
@@ -9003,7 +9296,7 @@
         <v>72</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>208</v>
+        <v>253</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>73</v>
@@ -9020,10 +9313,10 @@
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>209</v>
+        <v>256</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>209</v>
+        <v>256</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -9046,13 +9339,13 @@
         <v>72</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>210</v>
+        <v>257</v>
       </c>
       <c r="M77" t="s" s="2">
-        <v>210</v>
+        <v>258</v>
       </c>
       <c r="N77" s="2"/>
       <c r="O77" s="2"/>
@@ -9103,7 +9396,7 @@
         <v>72</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>209</v>
+        <v>256</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>73</v>
@@ -9120,10 +9413,10 @@
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>211</v>
+        <v>259</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>211</v>
+        <v>259</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -9149,10 +9442,10 @@
         <v>78</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>212</v>
+        <v>260</v>
       </c>
       <c r="M78" t="s" s="2">
-        <v>212</v>
+        <v>261</v>
       </c>
       <c r="N78" s="2"/>
       <c r="O78" s="2"/>
@@ -9203,7 +9496,7 @@
         <v>72</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>211</v>
+        <v>259</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>73</v>
@@ -9220,10 +9513,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>213</v>
+        <v>262</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>213</v>
+        <v>262</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -9320,10 +9613,10 @@
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>214</v>
+        <v>263</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>214</v>
+        <v>263</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -9422,10 +9715,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>215</v>
+        <v>264</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>215</v>
+        <v>264</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -9526,10 +9819,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>216</v>
+        <v>265</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>216</v>
+        <v>265</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -9555,10 +9848,10 @@
         <v>113</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>114</v>
+        <v>266</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>114</v>
+        <v>267</v>
       </c>
       <c r="N82" s="2"/>
       <c r="O82" s="2"/>
@@ -9609,7 +9902,7 @@
         <v>72</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>216</v>
+        <v>265</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>73</v>
@@ -9626,10 +9919,10 @@
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
-        <v>217</v>
+        <v>268</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>217</v>
+        <v>268</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -9652,13 +9945,13 @@
         <v>72</v>
       </c>
       <c r="K83" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>117</v>
+        <v>269</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>117</v>
+        <v>270</v>
       </c>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -9709,7 +10002,7 @@
         <v>72</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>217</v>
+        <v>268</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>83</v>
@@ -9726,10 +10019,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
-        <v>218</v>
+        <v>271</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>218</v>
+        <v>271</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -9755,10 +10048,10 @@
         <v>78</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>219</v>
+        <v>272</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>219</v>
+        <v>273</v>
       </c>
       <c r="N84" s="2"/>
       <c r="O84" s="2"/>
@@ -9809,7 +10102,7 @@
         <v>72</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>218</v>
+        <v>271</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>73</v>
@@ -9826,10 +10119,10 @@
     </row>
     <row r="85">
       <c r="A85" t="s" s="2">
-        <v>220</v>
+        <v>274</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>220</v>
+        <v>274</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -9926,10 +10219,10 @@
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>221</v>
+        <v>275</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>221</v>
+        <v>275</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -10028,10 +10321,10 @@
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>222</v>
+        <v>276</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>222</v>
+        <v>276</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -10132,10 +10425,10 @@
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>223</v>
+        <v>277</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>223</v>
+        <v>277</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -10158,13 +10451,13 @@
         <v>72</v>
       </c>
       <c r="K88" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>224</v>
+        <v>278</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>225</v>
+        <v>279</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -10215,7 +10508,7 @@
         <v>72</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>223</v>
+        <v>277</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>73</v>
@@ -10232,10 +10525,10 @@
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>226</v>
+        <v>280</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>226</v>
+        <v>280</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -10261,10 +10554,10 @@
         <v>78</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>227</v>
+        <v>281</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>227</v>
+        <v>282</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
@@ -10315,7 +10608,7 @@
         <v>72</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>226</v>
+        <v>280</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>83</v>
@@ -10332,10 +10625,10 @@
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>228</v>
+        <v>283</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>228</v>
+        <v>283</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -10432,10 +10725,10 @@
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>229</v>
+        <v>284</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>229</v>
+        <v>284</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -10534,10 +10827,10 @@
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>230</v>
+        <v>285</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>230</v>
+        <v>285</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -10638,10 +10931,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>231</v>
+        <v>286</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>231</v>
+        <v>286</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -10664,13 +10957,13 @@
         <v>72</v>
       </c>
       <c r="K93" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>210</v>
+        <v>287</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>210</v>
+        <v>288</v>
       </c>
       <c r="N93" s="2"/>
       <c r="O93" s="2"/>
@@ -10721,7 +11014,7 @@
         <v>72</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>231</v>
+        <v>286</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>83</v>
@@ -10738,10 +11031,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>232</v>
+        <v>289</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>232</v>
+        <v>289</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -10764,13 +11057,13 @@
         <v>72</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>176</v>
+        <v>290</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>233</v>
+        <v>291</v>
       </c>
       <c r="N94" s="2"/>
       <c r="O94" s="2"/>
@@ -10821,7 +11114,7 @@
         <v>72</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>232</v>
+        <v>289</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>73</v>
@@ -10838,10 +11131,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>234</v>
+        <v>292</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>234</v>
+        <v>292</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -10867,10 +11160,10 @@
         <v>78</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>235</v>
+        <v>293</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>235</v>
+        <v>294</v>
       </c>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -10921,7 +11214,7 @@
         <v>72</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>234</v>
+        <v>292</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>73</v>
@@ -10938,10 +11231,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>236</v>
+        <v>295</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>236</v>
+        <v>295</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -11038,10 +11331,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>237</v>
+        <v>296</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>237</v>
+        <v>296</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -11140,10 +11433,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>238</v>
+        <v>297</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>238</v>
+        <v>297</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -11244,10 +11537,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>239</v>
+        <v>298</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>239</v>
+        <v>298</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -11270,13 +11563,13 @@
         <v>72</v>
       </c>
       <c r="K99" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>224</v>
+        <v>299</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="N99" s="2"/>
       <c r="O99" s="2"/>
@@ -11327,7 +11620,7 @@
         <v>72</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>239</v>
+        <v>298</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>83</v>
@@ -11344,10 +11637,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -11370,13 +11663,13 @@
         <v>72</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>210</v>
+        <v>302</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>210</v>
+        <v>303</v>
       </c>
       <c r="N100" s="2"/>
       <c r="O100" s="2"/>
@@ -11427,7 +11720,7 @@
         <v>72</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>83</v>
@@ -11444,10 +11737,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>242</v>
+        <v>304</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>242</v>
+        <v>304</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -11473,10 +11766,10 @@
         <v>78</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>243</v>
+        <v>305</v>
       </c>
       <c r="M101" t="s" s="2">
-        <v>244</v>
+        <v>306</v>
       </c>
       <c r="N101" s="2"/>
       <c r="O101" s="2"/>
@@ -11527,7 +11820,7 @@
         <v>72</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>242</v>
+        <v>304</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>83</v>
@@ -11544,10 +11837,10 @@
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
-        <v>245</v>
+        <v>307</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>245</v>
+        <v>307</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -11644,10 +11937,10 @@
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>246</v>
+        <v>308</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>246</v>
+        <v>308</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -11746,10 +12039,10 @@
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
-        <v>247</v>
+        <v>309</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>247</v>
+        <v>309</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -11850,10 +12143,10 @@
     </row>
     <row r="105">
       <c r="A105" t="s" s="2">
-        <v>248</v>
+        <v>310</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>248</v>
+        <v>310</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -11879,10 +12172,10 @@
         <v>113</v>
       </c>
       <c r="L105" t="s" s="2">
-        <v>114</v>
+        <v>311</v>
       </c>
       <c r="M105" t="s" s="2">
-        <v>114</v>
+        <v>312</v>
       </c>
       <c r="N105" s="2"/>
       <c r="O105" s="2"/>
@@ -11933,7 +12226,7 @@
         <v>72</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>248</v>
+        <v>310</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>83</v>
@@ -11950,10 +12243,10 @@
     </row>
     <row r="106">
       <c r="A106" t="s" s="2">
-        <v>249</v>
+        <v>313</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>249</v>
+        <v>313</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -11979,10 +12272,10 @@
         <v>78</v>
       </c>
       <c r="L106" t="s" s="2">
-        <v>250</v>
+        <v>314</v>
       </c>
       <c r="M106" t="s" s="2">
-        <v>251</v>
+        <v>315</v>
       </c>
       <c r="N106" s="2"/>
       <c r="O106" s="2"/>
@@ -12033,7 +12326,7 @@
         <v>72</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>249</v>
+        <v>313</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>83</v>
@@ -12050,10 +12343,10 @@
     </row>
     <row r="107">
       <c r="A107" t="s" s="2">
-        <v>252</v>
+        <v>316</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>252</v>
+        <v>316</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -12150,10 +12443,10 @@
     </row>
     <row r="108">
       <c r="A108" t="s" s="2">
-        <v>253</v>
+        <v>317</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>253</v>
+        <v>317</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -12252,10 +12545,10 @@
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>254</v>
+        <v>318</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>254</v>
+        <v>318</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -12356,10 +12649,10 @@
     </row>
     <row r="110">
       <c r="A110" t="s" s="2">
-        <v>255</v>
+        <v>319</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>255</v>
+        <v>319</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -12385,10 +12678,10 @@
         <v>113</v>
       </c>
       <c r="L110" t="s" s="2">
-        <v>114</v>
+        <v>320</v>
       </c>
       <c r="M110" t="s" s="2">
-        <v>114</v>
+        <v>321</v>
       </c>
       <c r="N110" s="2"/>
       <c r="O110" s="2"/>
@@ -12439,7 +12732,7 @@
         <v>72</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>255</v>
+        <v>319</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>83</v>
@@ -12456,10 +12749,10 @@
     </row>
     <row r="111">
       <c r="A111" t="s" s="2">
-        <v>256</v>
+        <v>322</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>256</v>
+        <v>322</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -12482,13 +12775,13 @@
         <v>72</v>
       </c>
       <c r="K111" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>176</v>
+        <v>323</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>176</v>
+        <v>324</v>
       </c>
       <c r="N111" s="2"/>
       <c r="O111" s="2"/>
@@ -12539,7 +12832,7 @@
         <v>72</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>256</v>
+        <v>322</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>83</v>
@@ -12556,10 +12849,10 @@
     </row>
     <row r="112">
       <c r="A112" t="s" s="2">
-        <v>257</v>
+        <v>325</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>257</v>
+        <v>325</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -12570,7 +12863,7 @@
         <v>73</v>
       </c>
       <c r="G112" t="s" s="2">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="H112" t="s" s="2">
         <v>72</v>
@@ -12582,13 +12875,13 @@
         <v>72</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>258</v>
+        <v>326</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>258</v>
+        <v>327</v>
       </c>
       <c r="N112" s="2"/>
       <c r="O112" s="2"/>
@@ -12639,13 +12932,13 @@
         <v>72</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>257</v>
+        <v>325</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AH112" t="s" s="2">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="AI112" t="s" s="2">
         <v>72</v>
@@ -12656,10 +12949,10 @@
     </row>
     <row r="113">
       <c r="A113" t="s" s="2">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -12685,10 +12978,10 @@
         <v>78</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>181</v>
+        <v>329</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>182</v>
+        <v>330</v>
       </c>
       <c r="N113" s="2"/>
       <c r="O113" s="2"/>
@@ -12739,7 +13032,7 @@
         <v>72</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>83</v>
@@ -12756,10 +13049,10 @@
     </row>
     <row r="114">
       <c r="A114" t="s" s="2">
-        <v>260</v>
+        <v>331</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>260</v>
+        <v>331</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -12856,10 +13149,10 @@
     </row>
     <row r="115">
       <c r="A115" t="s" s="2">
-        <v>261</v>
+        <v>332</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>261</v>
+        <v>332</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -12958,10 +13251,10 @@
     </row>
     <row r="116">
       <c r="A116" t="s" s="2">
-        <v>262</v>
+        <v>333</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>262</v>
+        <v>333</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -13062,10 +13355,10 @@
     </row>
     <row r="117">
       <c r="A117" t="s" s="2">
-        <v>263</v>
+        <v>334</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>263</v>
+        <v>334</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -13088,13 +13381,13 @@
         <v>72</v>
       </c>
       <c r="K117" t="s" s="2">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="L117" t="s" s="2">
-        <v>165</v>
+        <v>335</v>
       </c>
       <c r="M117" t="s" s="2">
-        <v>165</v>
+        <v>335</v>
       </c>
       <c r="N117" s="2"/>
       <c r="O117" s="2"/>
@@ -13145,7 +13438,7 @@
         <v>72</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>263</v>
+        <v>334</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>73</v>
@@ -13162,10 +13455,10 @@
     </row>
     <row r="118">
       <c r="A118" t="s" s="2">
-        <v>264</v>
+        <v>336</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>264</v>
+        <v>336</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
@@ -13188,13 +13481,13 @@
         <v>72</v>
       </c>
       <c r="K118" t="s" s="2">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="L118" t="s" s="2">
-        <v>165</v>
+        <v>335</v>
       </c>
       <c r="M118" t="s" s="2">
-        <v>165</v>
+        <v>335</v>
       </c>
       <c r="N118" s="2"/>
       <c r="O118" s="2"/>
@@ -13245,7 +13538,7 @@
         <v>72</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>264</v>
+        <v>336</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>73</v>
@@ -13262,10 +13555,10 @@
     </row>
     <row r="119">
       <c r="A119" t="s" s="2">
-        <v>265</v>
+        <v>337</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>265</v>
+        <v>337</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" t="s" s="2">
@@ -13288,13 +13581,13 @@
         <v>72</v>
       </c>
       <c r="K119" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L119" t="s" s="2">
-        <v>266</v>
+        <v>338</v>
       </c>
       <c r="M119" t="s" s="2">
-        <v>266</v>
+        <v>339</v>
       </c>
       <c r="N119" s="2"/>
       <c r="O119" s="2"/>
@@ -13345,7 +13638,7 @@
         <v>72</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>265</v>
+        <v>337</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>73</v>
@@ -13362,10 +13655,10 @@
     </row>
     <row r="120">
       <c r="A120" t="s" s="2">
-        <v>267</v>
+        <v>340</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>267</v>
+        <v>340</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -13391,10 +13684,10 @@
         <v>78</v>
       </c>
       <c r="L120" t="s" s="2">
-        <v>210</v>
+        <v>341</v>
       </c>
       <c r="M120" t="s" s="2">
-        <v>210</v>
+        <v>342</v>
       </c>
       <c r="N120" s="2"/>
       <c r="O120" s="2"/>
@@ -13445,7 +13738,7 @@
         <v>72</v>
       </c>
       <c r="AF120" t="s" s="2">
-        <v>267</v>
+        <v>340</v>
       </c>
       <c r="AG120" t="s" s="2">
         <v>83</v>
@@ -13462,10 +13755,10 @@
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>268</v>
+        <v>343</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>268</v>
+        <v>343</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -13562,10 +13855,10 @@
     </row>
     <row r="122">
       <c r="A122" t="s" s="2">
-        <v>269</v>
+        <v>344</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>269</v>
+        <v>344</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -13664,10 +13957,10 @@
     </row>
     <row r="123">
       <c r="A123" t="s" s="2">
-        <v>270</v>
+        <v>345</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>270</v>
+        <v>345</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -13768,10 +14061,10 @@
     </row>
     <row r="124">
       <c r="A124" t="s" s="2">
-        <v>271</v>
+        <v>346</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>271</v>
+        <v>346</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -13794,13 +14087,13 @@
         <v>72</v>
       </c>
       <c r="K124" t="s" s="2">
-        <v>272</v>
+        <v>347</v>
       </c>
       <c r="L124" t="s" s="2">
-        <v>273</v>
+        <v>348</v>
       </c>
       <c r="M124" t="s" s="2">
-        <v>273</v>
+        <v>349</v>
       </c>
       <c r="N124" s="2"/>
       <c r="O124" s="2"/>
@@ -13851,7 +14144,7 @@
         <v>72</v>
       </c>
       <c r="AF124" t="s" s="2">
-        <v>271</v>
+        <v>346</v>
       </c>
       <c r="AG124" t="s" s="2">
         <v>73</v>
@@ -13868,10 +14161,10 @@
     </row>
     <row r="125">
       <c r="A125" t="s" s="2">
-        <v>274</v>
+        <v>350</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>274</v>
+        <v>350</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
@@ -13894,13 +14187,13 @@
         <v>72</v>
       </c>
       <c r="K125" t="s" s="2">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="L125" t="s" s="2">
-        <v>165</v>
+        <v>351</v>
       </c>
       <c r="M125" t="s" s="2">
-        <v>165</v>
+        <v>352</v>
       </c>
       <c r="N125" s="2"/>
       <c r="O125" s="2"/>
@@ -13951,7 +14244,7 @@
         <v>72</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>274</v>
+        <v>350</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>73</v>
@@ -13968,10 +14261,10 @@
     </row>
     <row r="126">
       <c r="A126" t="s" s="2">
-        <v>275</v>
+        <v>353</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>275</v>
+        <v>353</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -13997,10 +14290,10 @@
         <v>78</v>
       </c>
       <c r="L126" t="s" s="2">
-        <v>181</v>
+        <v>329</v>
       </c>
       <c r="M126" t="s" s="2">
-        <v>182</v>
+        <v>330</v>
       </c>
       <c r="N126" s="2"/>
       <c r="O126" s="2"/>
@@ -14051,7 +14344,7 @@
         <v>72</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>275</v>
+        <v>353</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>73</v>
@@ -14068,10 +14361,10 @@
     </row>
     <row r="127">
       <c r="A127" t="s" s="2">
-        <v>276</v>
+        <v>354</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>276</v>
+        <v>354</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -14168,10 +14461,10 @@
     </row>
     <row r="128">
       <c r="A128" t="s" s="2">
-        <v>277</v>
+        <v>355</v>
       </c>
       <c r="B128" t="s" s="2">
-        <v>277</v>
+        <v>355</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" t="s" s="2">
@@ -14270,10 +14563,10 @@
     </row>
     <row r="129">
       <c r="A129" t="s" s="2">
-        <v>278</v>
+        <v>356</v>
       </c>
       <c r="B129" t="s" s="2">
-        <v>278</v>
+        <v>356</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" t="s" s="2">
@@ -14374,10 +14667,10 @@
     </row>
     <row r="130">
       <c r="A130" t="s" s="2">
-        <v>279</v>
+        <v>357</v>
       </c>
       <c r="B130" t="s" s="2">
-        <v>279</v>
+        <v>357</v>
       </c>
       <c r="C130" s="2"/>
       <c r="D130" t="s" s="2">
@@ -14400,13 +14693,13 @@
         <v>72</v>
       </c>
       <c r="K130" t="s" s="2">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="L130" t="s" s="2">
-        <v>165</v>
+        <v>335</v>
       </c>
       <c r="M130" t="s" s="2">
-        <v>165</v>
+        <v>335</v>
       </c>
       <c r="N130" s="2"/>
       <c r="O130" s="2"/>
@@ -14457,7 +14750,7 @@
         <v>72</v>
       </c>
       <c r="AF130" t="s" s="2">
-        <v>279</v>
+        <v>357</v>
       </c>
       <c r="AG130" t="s" s="2">
         <v>73</v>
@@ -14474,10 +14767,10 @@
     </row>
     <row r="131">
       <c r="A131" t="s" s="2">
-        <v>280</v>
+        <v>358</v>
       </c>
       <c r="B131" t="s" s="2">
-        <v>280</v>
+        <v>358</v>
       </c>
       <c r="C131" s="2"/>
       <c r="D131" t="s" s="2">
@@ -14500,13 +14793,13 @@
         <v>72</v>
       </c>
       <c r="K131" t="s" s="2">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="L131" t="s" s="2">
-        <v>165</v>
+        <v>335</v>
       </c>
       <c r="M131" t="s" s="2">
-        <v>165</v>
+        <v>335</v>
       </c>
       <c r="N131" s="2"/>
       <c r="O131" s="2"/>
@@ -14557,7 +14850,7 @@
         <v>72</v>
       </c>
       <c r="AF131" t="s" s="2">
-        <v>280</v>
+        <v>358</v>
       </c>
       <c r="AG131" t="s" s="2">
         <v>73</v>
@@ -14574,10 +14867,10 @@
     </row>
     <row r="132">
       <c r="A132" t="s" s="2">
-        <v>281</v>
+        <v>359</v>
       </c>
       <c r="B132" t="s" s="2">
-        <v>281</v>
+        <v>359</v>
       </c>
       <c r="C132" s="2"/>
       <c r="D132" t="s" s="2">
@@ -14600,13 +14893,13 @@
         <v>72</v>
       </c>
       <c r="K132" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L132" t="s" s="2">
-        <v>282</v>
+        <v>360</v>
       </c>
       <c r="M132" t="s" s="2">
-        <v>282</v>
+        <v>361</v>
       </c>
       <c r="N132" s="2"/>
       <c r="O132" s="2"/>
@@ -14657,7 +14950,7 @@
         <v>72</v>
       </c>
       <c r="AF132" t="s" s="2">
-        <v>281</v>
+        <v>359</v>
       </c>
       <c r="AG132" t="s" s="2">
         <v>73</v>
@@ -14674,10 +14967,10 @@
     </row>
     <row r="133">
       <c r="A133" t="s" s="2">
-        <v>283</v>
+        <v>362</v>
       </c>
       <c r="B133" t="s" s="2">
-        <v>283</v>
+        <v>362</v>
       </c>
       <c r="C133" s="2"/>
       <c r="D133" t="s" s="2">
@@ -14700,13 +14993,13 @@
         <v>72</v>
       </c>
       <c r="K133" t="s" s="2">
-        <v>284</v>
+        <v>363</v>
       </c>
       <c r="L133" t="s" s="2">
-        <v>285</v>
+        <v>364</v>
       </c>
       <c r="M133" t="s" s="2">
-        <v>285</v>
+        <v>364</v>
       </c>
       <c r="N133" s="2"/>
       <c r="O133" s="2"/>
@@ -14757,7 +15050,7 @@
         <v>72</v>
       </c>
       <c r="AF133" t="s" s="2">
-        <v>283</v>
+        <v>362</v>
       </c>
       <c r="AG133" t="s" s="2">
         <v>73</v>
@@ -14774,10 +15067,10 @@
     </row>
     <row r="134">
       <c r="A134" t="s" s="2">
-        <v>286</v>
+        <v>365</v>
       </c>
       <c r="B134" t="s" s="2">
-        <v>286</v>
+        <v>365</v>
       </c>
       <c r="C134" s="2"/>
       <c r="D134" t="s" s="2">
@@ -14800,13 +15093,13 @@
         <v>72</v>
       </c>
       <c r="K134" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L134" t="s" s="2">
-        <v>287</v>
+        <v>366</v>
       </c>
       <c r="M134" t="s" s="2">
-        <v>287</v>
+        <v>367</v>
       </c>
       <c r="N134" s="2"/>
       <c r="O134" s="2"/>
@@ -14857,7 +15150,7 @@
         <v>72</v>
       </c>
       <c r="AF134" t="s" s="2">
-        <v>286</v>
+        <v>365</v>
       </c>
       <c r="AG134" t="s" s="2">
         <v>73</v>
@@ -14874,10 +15167,10 @@
     </row>
     <row r="135">
       <c r="A135" t="s" s="2">
-        <v>288</v>
+        <v>368</v>
       </c>
       <c r="B135" t="s" s="2">
-        <v>288</v>
+        <v>368</v>
       </c>
       <c r="C135" s="2"/>
       <c r="D135" t="s" s="2">
@@ -14900,13 +15193,13 @@
         <v>72</v>
       </c>
       <c r="K135" t="s" s="2">
-        <v>289</v>
+        <v>369</v>
       </c>
       <c r="L135" t="s" s="2">
-        <v>290</v>
+        <v>370</v>
       </c>
       <c r="M135" t="s" s="2">
-        <v>290</v>
+        <v>371</v>
       </c>
       <c r="N135" s="2"/>
       <c r="O135" s="2"/>
@@ -14957,7 +15250,7 @@
         <v>72</v>
       </c>
       <c r="AF135" t="s" s="2">
-        <v>288</v>
+        <v>368</v>
       </c>
       <c r="AG135" t="s" s="2">
         <v>83</v>
@@ -14974,10 +15267,10 @@
     </row>
     <row r="136">
       <c r="A136" t="s" s="2">
-        <v>291</v>
+        <v>372</v>
       </c>
       <c r="B136" t="s" s="2">
-        <v>291</v>
+        <v>372</v>
       </c>
       <c r="C136" s="2"/>
       <c r="D136" t="s" s="2">
@@ -15000,13 +15293,13 @@
         <v>72</v>
       </c>
       <c r="K136" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L136" t="s" s="2">
-        <v>292</v>
+        <v>373</v>
       </c>
       <c r="M136" t="s" s="2">
-        <v>292</v>
+        <v>374</v>
       </c>
       <c r="N136" s="2"/>
       <c r="O136" s="2"/>
@@ -15057,7 +15350,7 @@
         <v>72</v>
       </c>
       <c r="AF136" t="s" s="2">
-        <v>291</v>
+        <v>372</v>
       </c>
       <c r="AG136" t="s" s="2">
         <v>73</v>
@@ -15074,10 +15367,10 @@
     </row>
     <row r="137">
       <c r="A137" t="s" s="2">
-        <v>293</v>
+        <v>375</v>
       </c>
       <c r="B137" t="s" s="2">
-        <v>293</v>
+        <v>375</v>
       </c>
       <c r="C137" s="2"/>
       <c r="D137" t="s" s="2">
@@ -15100,13 +15393,13 @@
         <v>72</v>
       </c>
       <c r="K137" t="s" s="2">
-        <v>289</v>
+        <v>369</v>
       </c>
       <c r="L137" t="s" s="2">
-        <v>294</v>
+        <v>376</v>
       </c>
       <c r="M137" t="s" s="2">
-        <v>294</v>
+        <v>377</v>
       </c>
       <c r="N137" s="2"/>
       <c r="O137" s="2"/>
@@ -15157,7 +15450,7 @@
         <v>72</v>
       </c>
       <c r="AF137" t="s" s="2">
-        <v>293</v>
+        <v>375</v>
       </c>
       <c r="AG137" t="s" s="2">
         <v>83</v>
@@ -15174,10 +15467,10 @@
     </row>
     <row r="138">
       <c r="A138" t="s" s="2">
-        <v>295</v>
+        <v>378</v>
       </c>
       <c r="B138" t="s" s="2">
-        <v>295</v>
+        <v>378</v>
       </c>
       <c r="C138" s="2"/>
       <c r="D138" t="s" s="2">
@@ -15200,13 +15493,13 @@
         <v>72</v>
       </c>
       <c r="K138" t="s" s="2">
-        <v>296</v>
+        <v>379</v>
       </c>
       <c r="L138" t="s" s="2">
-        <v>297</v>
+        <v>380</v>
       </c>
       <c r="M138" t="s" s="2">
-        <v>298</v>
+        <v>381</v>
       </c>
       <c r="N138" s="2"/>
       <c r="O138" s="2"/>
@@ -15257,7 +15550,7 @@
         <v>72</v>
       </c>
       <c r="AF138" t="s" s="2">
-        <v>295</v>
+        <v>378</v>
       </c>
       <c r="AG138" t="s" s="2">
         <v>73</v>
@@ -15274,10 +15567,10 @@
     </row>
     <row r="139">
       <c r="A139" t="s" s="2">
-        <v>299</v>
+        <v>382</v>
       </c>
       <c r="B139" t="s" s="2">
-        <v>299</v>
+        <v>382</v>
       </c>
       <c r="C139" s="2"/>
       <c r="D139" t="s" s="2">
@@ -15303,10 +15596,10 @@
         <v>78</v>
       </c>
       <c r="L139" t="s" s="2">
-        <v>300</v>
+        <v>383</v>
       </c>
       <c r="M139" t="s" s="2">
-        <v>300</v>
+        <v>384</v>
       </c>
       <c r="N139" s="2"/>
       <c r="O139" s="2"/>
@@ -15357,7 +15650,7 @@
         <v>72</v>
       </c>
       <c r="AF139" t="s" s="2">
-        <v>299</v>
+        <v>382</v>
       </c>
       <c r="AG139" t="s" s="2">
         <v>73</v>
@@ -15374,10 +15667,10 @@
     </row>
     <row r="140">
       <c r="A140" t="s" s="2">
-        <v>301</v>
+        <v>385</v>
       </c>
       <c r="B140" t="s" s="2">
-        <v>301</v>
+        <v>385</v>
       </c>
       <c r="C140" s="2"/>
       <c r="D140" t="s" s="2">
@@ -15474,10 +15767,10 @@
     </row>
     <row r="141">
       <c r="A141" t="s" s="2">
-        <v>302</v>
+        <v>386</v>
       </c>
       <c r="B141" t="s" s="2">
-        <v>302</v>
+        <v>386</v>
       </c>
       <c r="C141" s="2"/>
       <c r="D141" t="s" s="2">
@@ -15576,10 +15869,10 @@
     </row>
     <row r="142">
       <c r="A142" t="s" s="2">
-        <v>303</v>
+        <v>387</v>
       </c>
       <c r="B142" t="s" s="2">
-        <v>303</v>
+        <v>387</v>
       </c>
       <c r="C142" s="2"/>
       <c r="D142" t="s" s="2">
@@ -15680,10 +15973,10 @@
     </row>
     <row r="143">
       <c r="A143" t="s" s="2">
-        <v>304</v>
+        <v>388</v>
       </c>
       <c r="B143" t="s" s="2">
-        <v>304</v>
+        <v>388</v>
       </c>
       <c r="C143" s="2"/>
       <c r="D143" t="s" s="2">
@@ -15706,13 +15999,13 @@
         <v>72</v>
       </c>
       <c r="K143" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L143" t="s" s="2">
-        <v>134</v>
+        <v>389</v>
       </c>
       <c r="M143" t="s" s="2">
-        <v>134</v>
+        <v>390</v>
       </c>
       <c r="N143" s="2"/>
       <c r="O143" s="2"/>
@@ -15763,7 +16056,7 @@
         <v>72</v>
       </c>
       <c r="AF143" t="s" s="2">
-        <v>304</v>
+        <v>388</v>
       </c>
       <c r="AG143" t="s" s="2">
         <v>83</v>
@@ -15780,10 +16073,10 @@
     </row>
     <row r="144">
       <c r="A144" t="s" s="2">
-        <v>305</v>
+        <v>391</v>
       </c>
       <c r="B144" t="s" s="2">
-        <v>305</v>
+        <v>391</v>
       </c>
       <c r="C144" s="2"/>
       <c r="D144" t="s" s="2">
@@ -15809,10 +16102,10 @@
         <v>78</v>
       </c>
       <c r="L144" t="s" s="2">
-        <v>306</v>
+        <v>392</v>
       </c>
       <c r="M144" t="s" s="2">
-        <v>306</v>
+        <v>393</v>
       </c>
       <c r="N144" s="2"/>
       <c r="O144" s="2"/>
@@ -15863,7 +16156,7 @@
         <v>72</v>
       </c>
       <c r="AF144" t="s" s="2">
-        <v>305</v>
+        <v>391</v>
       </c>
       <c r="AG144" t="s" s="2">
         <v>83</v>
@@ -15880,10 +16173,10 @@
     </row>
     <row r="145">
       <c r="A145" t="s" s="2">
-        <v>307</v>
+        <v>394</v>
       </c>
       <c r="B145" t="s" s="2">
-        <v>307</v>
+        <v>394</v>
       </c>
       <c r="C145" s="2"/>
       <c r="D145" t="s" s="2">
@@ -15980,10 +16273,10 @@
     </row>
     <row r="146">
       <c r="A146" t="s" s="2">
-        <v>308</v>
+        <v>395</v>
       </c>
       <c r="B146" t="s" s="2">
-        <v>308</v>
+        <v>395</v>
       </c>
       <c r="C146" s="2"/>
       <c r="D146" t="s" s="2">
@@ -16082,10 +16375,10 @@
     </row>
     <row r="147">
       <c r="A147" t="s" s="2">
-        <v>309</v>
+        <v>396</v>
       </c>
       <c r="B147" t="s" s="2">
-        <v>309</v>
+        <v>396</v>
       </c>
       <c r="C147" s="2"/>
       <c r="D147" t="s" s="2">
@@ -16186,10 +16479,10 @@
     </row>
     <row r="148">
       <c r="A148" t="s" s="2">
-        <v>310</v>
+        <v>397</v>
       </c>
       <c r="B148" t="s" s="2">
-        <v>310</v>
+        <v>397</v>
       </c>
       <c r="C148" s="2"/>
       <c r="D148" t="s" s="2">
@@ -16215,10 +16508,10 @@
         <v>113</v>
       </c>
       <c r="L148" t="s" s="2">
-        <v>114</v>
+        <v>398</v>
       </c>
       <c r="M148" t="s" s="2">
-        <v>114</v>
+        <v>399</v>
       </c>
       <c r="N148" s="2"/>
       <c r="O148" s="2"/>
@@ -16269,7 +16562,7 @@
         <v>72</v>
       </c>
       <c r="AF148" t="s" s="2">
-        <v>310</v>
+        <v>397</v>
       </c>
       <c r="AG148" t="s" s="2">
         <v>83</v>
@@ -16286,10 +16579,10 @@
     </row>
     <row r="149">
       <c r="A149" t="s" s="2">
-        <v>311</v>
+        <v>400</v>
       </c>
       <c r="B149" t="s" s="2">
-        <v>311</v>
+        <v>400</v>
       </c>
       <c r="C149" s="2"/>
       <c r="D149" t="s" s="2">
@@ -16312,13 +16605,13 @@
         <v>72</v>
       </c>
       <c r="K149" t="s" s="2">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="L149" t="s" s="2">
-        <v>165</v>
+        <v>401</v>
       </c>
       <c r="M149" t="s" s="2">
-        <v>165</v>
+        <v>402</v>
       </c>
       <c r="N149" s="2"/>
       <c r="O149" s="2"/>
@@ -16369,7 +16662,7 @@
         <v>72</v>
       </c>
       <c r="AF149" t="s" s="2">
-        <v>311</v>
+        <v>400</v>
       </c>
       <c r="AG149" t="s" s="2">
         <v>83</v>
@@ -16386,10 +16679,10 @@
     </row>
     <row r="150">
       <c r="A150" t="s" s="2">
-        <v>312</v>
+        <v>403</v>
       </c>
       <c r="B150" t="s" s="2">
-        <v>312</v>
+        <v>403</v>
       </c>
       <c r="C150" s="2"/>
       <c r="D150" t="s" s="2">
@@ -16412,13 +16705,13 @@
         <v>72</v>
       </c>
       <c r="K150" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L150" t="s" s="2">
-        <v>176</v>
+        <v>404</v>
       </c>
       <c r="M150" t="s" s="2">
-        <v>176</v>
+        <v>405</v>
       </c>
       <c r="N150" s="2"/>
       <c r="O150" s="2"/>
@@ -16469,7 +16762,7 @@
         <v>72</v>
       </c>
       <c r="AF150" t="s" s="2">
-        <v>312</v>
+        <v>403</v>
       </c>
       <c r="AG150" t="s" s="2">
         <v>83</v>
@@ -16486,10 +16779,10 @@
     </row>
     <row r="151">
       <c r="A151" t="s" s="2">
-        <v>313</v>
+        <v>406</v>
       </c>
       <c r="B151" t="s" s="2">
-        <v>313</v>
+        <v>406</v>
       </c>
       <c r="C151" s="2"/>
       <c r="D151" t="s" s="2">
@@ -16515,10 +16808,10 @@
         <v>78</v>
       </c>
       <c r="L151" t="s" s="2">
-        <v>314</v>
+        <v>407</v>
       </c>
       <c r="M151" t="s" s="2">
-        <v>314</v>
+        <v>408</v>
       </c>
       <c r="N151" s="2"/>
       <c r="O151" s="2"/>
@@ -16569,7 +16862,7 @@
         <v>72</v>
       </c>
       <c r="AF151" t="s" s="2">
-        <v>313</v>
+        <v>406</v>
       </c>
       <c r="AG151" t="s" s="2">
         <v>83</v>
@@ -16586,10 +16879,10 @@
     </row>
     <row r="152">
       <c r="A152" t="s" s="2">
-        <v>315</v>
+        <v>409</v>
       </c>
       <c r="B152" t="s" s="2">
-        <v>315</v>
+        <v>409</v>
       </c>
       <c r="C152" s="2"/>
       <c r="D152" t="s" s="2">
@@ -16686,10 +16979,10 @@
     </row>
     <row r="153">
       <c r="A153" t="s" s="2">
-        <v>316</v>
+        <v>410</v>
       </c>
       <c r="B153" t="s" s="2">
-        <v>316</v>
+        <v>410</v>
       </c>
       <c r="C153" s="2"/>
       <c r="D153" t="s" s="2">
@@ -16788,10 +17081,10 @@
     </row>
     <row r="154">
       <c r="A154" t="s" s="2">
-        <v>317</v>
+        <v>411</v>
       </c>
       <c r="B154" t="s" s="2">
-        <v>317</v>
+        <v>411</v>
       </c>
       <c r="C154" s="2"/>
       <c r="D154" t="s" s="2">
@@ -16892,10 +17185,10 @@
     </row>
     <row r="155">
       <c r="A155" t="s" s="2">
-        <v>318</v>
+        <v>412</v>
       </c>
       <c r="B155" t="s" s="2">
-        <v>318</v>
+        <v>412</v>
       </c>
       <c r="C155" s="2"/>
       <c r="D155" t="s" s="2">
@@ -16921,10 +17214,10 @@
         <v>113</v>
       </c>
       <c r="L155" t="s" s="2">
-        <v>114</v>
+        <v>413</v>
       </c>
       <c r="M155" t="s" s="2">
-        <v>114</v>
+        <v>414</v>
       </c>
       <c r="N155" s="2"/>
       <c r="O155" s="2"/>
@@ -16975,7 +17268,7 @@
         <v>72</v>
       </c>
       <c r="AF155" t="s" s="2">
-        <v>318</v>
+        <v>412</v>
       </c>
       <c r="AG155" t="s" s="2">
         <v>83</v>

</xml_diff>